<commit_message>
Fix: labels categorias SONY ONE/IBERIA, sufijo min en UI, COMERCIALES minutos totales
</commit_message>
<xml_diff>
--- a/import_versions.xlsx
+++ b/import_versions.xlsx
@@ -397,10 +397,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:D68"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -410,6 +412,12 @@
       <c r="B1" t="str">
         <v>category</v>
       </c>
+      <c r="C1" t="str">
+        <v>platform</v>
+      </c>
+      <c r="D1" t="str">
+        <v>duration</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -418,6 +426,12 @@
       <c r="B2" t="str">
         <v/>
       </c>
+      <c r="C2" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -426,6 +440,12 @@
       <c r="B3" t="str">
         <v/>
       </c>
+      <c r="C3" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -434,6 +454,12 @@
       <c r="B4" t="str">
         <v/>
       </c>
+      <c r="C4" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -442,6 +468,12 @@
       <c r="B5" t="str">
         <v/>
       </c>
+      <c r="C5" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -450,6 +482,12 @@
       <c r="B6" t="str">
         <v/>
       </c>
+      <c r="C6" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -458,6 +496,12 @@
       <c r="B7" t="str">
         <v/>
       </c>
+      <c r="C7" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -466,6 +510,12 @@
       <c r="B8" t="str">
         <v/>
       </c>
+      <c r="C8" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -474,6 +524,12 @@
       <c r="B9" t="str">
         <v/>
       </c>
+      <c r="C9" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -482,6 +538,12 @@
       <c r="B10" t="str">
         <v/>
       </c>
+      <c r="C10" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -490,6 +552,12 @@
       <c r="B11" t="str">
         <v/>
       </c>
+      <c r="C11" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -498,6 +566,12 @@
       <c r="B12" t="str">
         <v/>
       </c>
+      <c r="C12" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -506,6 +580,12 @@
       <c r="B13" t="str">
         <v/>
       </c>
+      <c r="C13" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -514,6 +594,12 @@
       <c r="B14" t="str">
         <v/>
       </c>
+      <c r="C14" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -522,6 +608,12 @@
       <c r="B15" t="str">
         <v/>
       </c>
+      <c r="C15" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -530,6 +622,12 @@
       <c r="B16" t="str">
         <v/>
       </c>
+      <c r="C16" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -538,6 +636,12 @@
       <c r="B17" t="str">
         <v/>
       </c>
+      <c r="C17" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -546,6 +650,12 @@
       <c r="B18" t="str">
         <v/>
       </c>
+      <c r="C18" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -554,6 +664,12 @@
       <c r="B19" t="str">
         <v/>
       </c>
+      <c r="C19" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -562,6 +678,12 @@
       <c r="B20" t="str">
         <v/>
       </c>
+      <c r="C20" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -570,6 +692,12 @@
       <c r="B21" t="str">
         <v/>
       </c>
+      <c r="C21" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -578,6 +706,12 @@
       <c r="B22" t="str">
         <v/>
       </c>
+      <c r="C22" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -586,6 +720,12 @@
       <c r="B23" t="str">
         <v/>
       </c>
+      <c r="C23" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -594,6 +734,12 @@
       <c r="B24" t="str">
         <v/>
       </c>
+      <c r="C24" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -602,6 +748,12 @@
       <c r="B25" t="str">
         <v/>
       </c>
+      <c r="C25" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -610,6 +762,12 @@
       <c r="B26" t="str">
         <v/>
       </c>
+      <c r="C26" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -618,6 +776,12 @@
       <c r="B27" t="str">
         <v/>
       </c>
+      <c r="C27" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -626,6 +790,12 @@
       <c r="B28" t="str">
         <v/>
       </c>
+      <c r="C28" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -634,6 +804,12 @@
       <c r="B29" t="str">
         <v/>
       </c>
+      <c r="C29" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -642,6 +818,12 @@
       <c r="B30" t="str">
         <v/>
       </c>
+      <c r="C30" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -650,6 +832,12 @@
       <c r="B31" t="str">
         <v/>
       </c>
+      <c r="C31" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -658,6 +846,12 @@
       <c r="B32" t="str">
         <v/>
       </c>
+      <c r="C32" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -666,6 +860,12 @@
       <c r="B33" t="str">
         <v/>
       </c>
+      <c r="C33" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -674,6 +874,12 @@
       <c r="B34" t="str">
         <v/>
       </c>
+      <c r="C34" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -682,6 +888,12 @@
       <c r="B35" t="str">
         <v/>
       </c>
+      <c r="C35" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -690,6 +902,12 @@
       <c r="B36" t="str">
         <v/>
       </c>
+      <c r="C36" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -698,6 +916,12 @@
       <c r="B37" t="str">
         <v/>
       </c>
+      <c r="C37" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -706,6 +930,12 @@
       <c r="B38" t="str">
         <v/>
       </c>
+      <c r="C38" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -714,6 +944,12 @@
       <c r="B39" t="str">
         <v/>
       </c>
+      <c r="C39" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -722,6 +958,12 @@
       <c r="B40" t="str">
         <v/>
       </c>
+      <c r="C40" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -730,6 +972,12 @@
       <c r="B41" t="str">
         <v/>
       </c>
+      <c r="C41" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -738,6 +986,12 @@
       <c r="B42" t="str">
         <v/>
       </c>
+      <c r="C42" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -746,6 +1000,12 @@
       <c r="B43" t="str">
         <v/>
       </c>
+      <c r="C43" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -754,6 +1014,12 @@
       <c r="B44" t="str">
         <v/>
       </c>
+      <c r="C44" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -762,6 +1028,12 @@
       <c r="B45" t="str">
         <v/>
       </c>
+      <c r="C45" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -770,6 +1042,12 @@
       <c r="B46" t="str">
         <v/>
       </c>
+      <c r="C46" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -778,6 +1056,12 @@
       <c r="B47" t="str">
         <v/>
       </c>
+      <c r="C47" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -786,6 +1070,12 @@
       <c r="B48" t="str">
         <v/>
       </c>
+      <c r="C48" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -794,6 +1084,12 @@
       <c r="B49" t="str">
         <v/>
       </c>
+      <c r="C49" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -802,6 +1098,12 @@
       <c r="B50" t="str">
         <v/>
       </c>
+      <c r="C50" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -810,6 +1112,12 @@
       <c r="B51" t="str">
         <v/>
       </c>
+      <c r="C51" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -818,6 +1126,12 @@
       <c r="B52" t="str">
         <v/>
       </c>
+      <c r="C52" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -826,6 +1140,12 @@
       <c r="B53" t="str">
         <v/>
       </c>
+      <c r="C53" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -834,6 +1154,12 @@
       <c r="B54" t="str">
         <v/>
       </c>
+      <c r="C54" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -842,6 +1168,12 @@
       <c r="B55" t="str">
         <v/>
       </c>
+      <c r="C55" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -850,6 +1182,12 @@
       <c r="B56" t="str">
         <v/>
       </c>
+      <c r="C56" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -858,6 +1196,12 @@
       <c r="B57" t="str">
         <v/>
       </c>
+      <c r="C57" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -866,6 +1210,12 @@
       <c r="B58" t="str">
         <v/>
       </c>
+      <c r="C58" t="str">
+        <v>LATAM</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -874,82 +1224,142 @@
       <c r="B59" t="str">
         <v/>
       </c>
+      <c r="C59" t="str">
+        <v>BRAZIL</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>e- FCHD1BSubtOpSCr</v>
+        <v>e- F HD4Bsubt-OpSCr</v>
       </c>
       <c r="B60" t="str">
         <v/>
+      </c>
+      <c r="C60" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D60">
+        <v>60</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>p- F HD Ci5BAFRISCr</v>
+        <v>p- FHD4BVOAFRISCTUR</v>
       </c>
       <c r="B61" t="str">
         <v/>
+      </c>
+      <c r="C61" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D61">
+        <v>60</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>p- FHD5BlocuAFRISCr</v>
+        <v>p- FHD4BVOAFRISCr</v>
       </c>
       <c r="B62" t="str">
         <v/>
+      </c>
+      <c r="C62" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D62">
+        <v>60</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>p- F HD Ci6BAFRISCr</v>
+        <v>e- FHD4Bsubt-OpSCAD</v>
       </c>
       <c r="B63" t="str">
         <v/>
+      </c>
+      <c r="C63" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D63">
+        <v>60</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>e- FCHD1BSubt-OpSCr</v>
+        <v>e- FCHD1BSubtOpSCr</v>
       </c>
       <c r="B64" t="str">
         <v/>
+      </c>
+      <c r="C64" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D64">
+        <v>120</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>e- F HD4Bsubt-OpSCr</v>
+        <v>p- F HD Ci5BAFRISCr</v>
       </c>
       <c r="B65" t="str">
         <v/>
+      </c>
+      <c r="C65" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D65">
+        <v>120</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>p- FHD4BVOAFRISCTUR</v>
+        <v>p- FHD5BlocuAFRISCr</v>
       </c>
       <c r="B66" t="str">
         <v/>
+      </c>
+      <c r="C66" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D66">
+        <v>120</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>p- FHD4BVOAFRISCr</v>
+        <v>p- F HD Ci6BAFRISCr</v>
       </c>
       <c r="B67" t="str">
         <v/>
+      </c>
+      <c r="C67" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D67">
+        <v>120</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>e- FHD4Bsubt-OpSCAD</v>
+        <v>e- FCHD1BSubt-OpSCr</v>
       </c>
       <c r="B68" t="str">
         <v/>
+      </c>
+      <c r="C68" t="str">
+        <v>IBERIA</v>
+      </c>
+      <c r="D68">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D68"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>